<commit_message>
feat: integrate interactive FlowButton component across site, create components/ui tsx files, and elevate layout
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,7 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="46" customWidth="1" min="12" max="12"/>
@@ -713,6 +713,74 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SG-261010180305</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 18:03:05</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Priya Rao</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>9848011223</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>priya.rao@example.com</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Inter BiPC (NEET Integrated)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2027-28</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada Girls Campus</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>FlowButton Integration Test</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>AI Chatbot Registration</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Pending Followup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sync enquiry logs and data records
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -490,14 +490,14 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="41" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="84" customWidth="1" min="12" max="12"/>
+    <col width="31" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -781,6 +781,74 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>SG-261010193527</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-10 19:35:27</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>testing@gmail.com</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Vijayawada (NTR Dist), Andhra Pradesh</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>BRAHMOS: IPE + NEET Medical (Bi.P.C)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2026 - 2027</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Residential (AC Class / Non-AC Hostel)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Class: Class 11 / Inter 1st Year | Campus: Residential (AC Class / Non-AC Hostel)</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>Admissions Page Enquiry Form</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Pending Followup</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: complete overhaul of AI Admissions Chatbot, add serverless api endpoints, verified institutional knowledge, and update favicon to official emblem
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -849,6 +849,222 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: embed critical scroller CSS inline, bust Safari favicon cache with SVG & unique filenames, and disable dev cache in server
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1065,78 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: integrate Google Sheets for website admission forms and AI chatbot enquiries
</commit_message>
<xml_diff>
--- a/enquiries.xlsx
+++ b/enquiries.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -493,7 +493,7 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="41" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="84" customWidth="1" min="12" max="12"/>
@@ -1137,6 +1137,282 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>SG-261013123731</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-13 12:37:31</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Aarav Varma</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>9849012345</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>aarav.varma@gmail.com</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Vijayawada (NTR Dist)</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>BRAHMOS: IPE + NEET Medical (Bi.P.C)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>2026 - 2027</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Residential (A/C Class + Non-A/C Hostel + Food)</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Admissions Enquiry</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Website Form</t>
+        </is>
+      </c>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SG-261013123747</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 12:37:47</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Keerthi Priya</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>9171222333</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>BRAHMOS: IPE + NEET Medical (Bi.P.C)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026 - 2027</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Residential Hostels</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Admissions Enquiry</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>AI Chatbot</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>SG-TEST999</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-11 11:30:00</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Test Student</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>9848012345</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>test@test.com</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Vijayawada</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Brahmos</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Hostel</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Test Suite</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>